<commit_message>
Atualização ASVS5.0 - Session management Documentation
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardorafaelnunessampaio/Documents/Docs/Mestrado/1o ano/2o Semestre/Desenvolvimento Soft Sec/Repo/Deliverables/Phase1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardorafaelnunessampaio/Documents/Docs/Mestrado/1o ano/2o Semestre/Desenvolvimento Soft Sec/Repo/Deliverables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34AED6A8-CA92-EE4D-A1FB-AB54BDFCE72C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF910935-E5C2-DB45-9408-1ECE3CBB70F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" tabRatio="500" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2072" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2074" uniqueCount="909">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2783,6 +2783,15 @@
   </si>
   <si>
     <t>Relatório, Secção "Conformidade com ASVS 5.0", Sub-secção "Validação de Inputs e lógica de negócio" v2.1.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relatório, Secção "Conformidade com ASVS 5.0", Sub-secção"Gestão de Sessões"  v7.1.1 </t>
+  </si>
+  <si>
+    <t>Relatório, Secção "Conformidade com ASVS 5.0", Sub-secção"Gestão de Sessões"  v7.1.2</t>
+  </si>
+  <si>
+    <t>Not Applicable</t>
   </si>
 </sst>
 </file>
@@ -3438,7 +3447,7 @@
                   <c:v>4.5454545454545456E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.16666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -3803,7 +3812,7 @@
                   <c:v>8.5106382978723402E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.10526315789473684</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -4759,11 +4768,11 @@
       </c>
       <c r="G12" s="4">
         <f>COUNTIFS('V7 - Session Management'!$F$2:$F$26,"Compliant",'V7 - Session Management'!$E$2:$E$26,2)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="I12" s="4">
         <v>1</v>
@@ -4778,11 +4787,11 @@
       </c>
       <c r="L12" s="4">
         <f>COUNTIF('V7 - Session Management'!$F$2:$F$26,"Compliant")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M12" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.10526315789473684</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -5295,11 +5304,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>1.948051948051948E-2</v>
+        <v>2.9284441049146931E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5315,11 +5324,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>2.7630692211418121E-2</v>
+        <v>3.3822642675814404E-2</v>
       </c>
     </row>
   </sheetData>
@@ -14306,10 +14315,12 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+      <c r="H3" s="16" t="s">
+        <v>906</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
@@ -14328,10 +14339,12 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
+        <v>893</v>
       </c>
       <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+      <c r="H4" s="21" t="s">
+        <v>907</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
@@ -14350,7 +14363,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
+        <v>908</v>
       </c>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>

</xml_diff>

<commit_message>
Ajustes de compliance com JWT para ASVS 5.0
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/ASVS_5.0_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardorafaelnunessampaio/Documents/Docs/Mestrado/1o ano/2o Semestre/Desenvolvimento Soft Sec/Repo/Deliverables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF910935-E5C2-DB45-9408-1ECE3CBB70F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99133BD2-2475-5948-AED5-286972AC992C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" tabRatio="500" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2074" uniqueCount="909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="916">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2792,6 +2792,30 @@
   </si>
   <si>
     <t>Not Applicable</t>
+  </si>
+  <si>
+    <t>Flask-JWT-Extended faz a a validação automática, a geração de signatures é feita através de secret keys</t>
+  </si>
+  <si>
+    <t>Fihceiro app.py:       app.config["JWT_SECRET_KEY"] = os.getenv("JWT_SECRET_KEY")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ficherio app.py:   app.config["JWT_DECODE_ALGORITHMS"] = ["HS256"]  </t>
+  </si>
+  <si>
+    <t>Flask-JWT-Extended permite a definição de allow list de algoritmos</t>
+  </si>
+  <si>
+    <t>O Flask-JWT-Extended com HS256 não é vulnerável a este ataque porque não usa chaves públicas</t>
+  </si>
+  <si>
+    <t>Ficheiro app.py: app.config["JWT_ACCESS_TOKEN_EXPIRES"] = timedelta(minutes=15)
+app.config["JWT_REFRESH_TOKEN_EXPIRES"] = timedelta(days=30)
+# verificação de nbf
+app.config["JWT_DECODE_LEEWAY"] = 0</t>
+  </si>
+  <si>
+    <t>Flask-JWT-Extended valida exp e nbf automaticamente através da definição dos seguintes parametros:</t>
   </si>
 </sst>
 </file>
@@ -3269,7 +3293,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -3818,7 +3842,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.5714285714285714</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -4855,11 +4879,11 @@
       </c>
       <c r="D14" s="4">
         <f>COUNTIFS('V9 - Self-contained Tokens'!$F$2:$F$10,"Compliant",'V9 - Self-contained Tokens'!$E$2:$E$10,1)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E14" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="4">
         <v>3</v>
@@ -4883,11 +4907,11 @@
       </c>
       <c r="L14" s="4">
         <f>COUNTIF('V9 - Self-contained Tokens'!$F$2:$F$10,"Compliant")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M14" s="5">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -5292,11 +5316,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>6.5384615384615388E-2</v>
+        <v>0.13205128205128205</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5324,11 +5348,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>3.3822642675814404E-2</v>
+        <v>6.7436088053965657E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5463,10 +5487,14 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+        <v>893</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>909</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>910</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
@@ -5485,10 +5513,14 @@
         <v>1</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+        <v>893</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>912</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>911</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
@@ -5507,10 +5539,14 @@
         <v>1</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
+        <v>893</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>913</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>911</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
@@ -5543,10 +5579,14 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+        <v>893</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>915</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>914</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="19" t="s">

</xml_diff>